<commit_message>
Add Pb-Free Solder Material and update the auto generating validating file
</commit_message>
<xml_diff>
--- a/data/raw/RPi_4_BoM_Official.xlsx
+++ b/data/raw/RPi_4_BoM_Official.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\szb75\Documents\Other_Proj\ArchitecturalCarbonModelingTool\ACT\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90469341-13BA-4C8D-B3E4-34417489014B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CADF8567-F811-4774-85EC-7EA34ADF0BC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-1575" yWindow="-18120" windowWidth="29040" windowHeight="17520" xr2:uid="{5023E1F4-0389-4A9C-A1C1-8A547001B1C6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{5023E1F4-0389-4A9C-A1C1-8A547001B1C6}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -88,7 +88,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="245">
   <si>
     <t>Quantity</t>
   </si>
@@ -811,6 +811,18 @@
   </si>
   <si>
     <t xml:space="preserve">Type </t>
+  </si>
+  <si>
+    <t>lpddr2_20nm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capacity </t>
+  </si>
+  <si>
+    <t>Process</t>
+  </si>
+  <si>
+    <t>pb free solder</t>
   </si>
 </sst>
 </file>
@@ -1584,7 +1596,7 @@
         <v>16</v>
       </c>
       <c r="T1" s="65" t="s">
-        <v>13</v>
+        <v>242</v>
       </c>
       <c r="U1" s="66" t="s">
         <v>14</v>
@@ -1595,7 +1607,9 @@
       <c r="W1" s="67" t="s">
         <v>240</v>
       </c>
-      <c r="X1" s="6"/>
+      <c r="X1" s="6" t="s">
+        <v>243</v>
+      </c>
       <c r="Y1" s="7"/>
       <c r="AB1" s="8"/>
       <c r="AC1" s="8"/>
@@ -1640,6 +1654,9 @@
       </c>
       <c r="U2" s="50">
         <v>159</v>
+      </c>
+      <c r="X2" t="s">
+        <v>241</v>
       </c>
       <c r="AB2" s="7"/>
       <c r="AC2" s="15"/>
@@ -1874,6 +1891,9 @@
       <c r="Q9" s="21"/>
       <c r="R9" s="21"/>
       <c r="S9" s="21"/>
+      <c r="W9" t="s">
+        <v>244</v>
+      </c>
       <c r="AB9" s="7"/>
       <c r="AC9" s="15"/>
       <c r="AD9" s="15"/>
@@ -2310,7 +2330,7 @@
       <c r="R22" s="21"/>
       <c r="S22" s="21"/>
     </row>
-    <row r="23" spans="2:35" ht="39.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="2:35" ht="27" x14ac:dyDescent="0.45">
       <c r="B23" s="17">
         <v>1</v>
       </c>
@@ -2444,7 +2464,7 @@
       <c r="AD26" s="15"/>
       <c r="AE26" s="15"/>
     </row>
-    <row r="27" spans="2:35" ht="51" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:35" ht="38.5" x14ac:dyDescent="0.35">
       <c r="B27" s="17">
         <v>1</v>
       </c>
@@ -2807,7 +2827,7 @@
       <c r="R38" s="21"/>
       <c r="S38" s="21"/>
     </row>
-    <row r="39" spans="2:31" ht="38.5" x14ac:dyDescent="0.35">
+    <row r="39" spans="2:31" ht="26" x14ac:dyDescent="0.35">
       <c r="B39" s="17">
         <v>1</v>
       </c>

</xml_diff>